<commit_message>
Corrige performance: busca so D-1 por dia e acumula historico em JSON
Antes, tanto PICKUP quanto DROPOFF reprocessavam o mes inteiro (dia 1 ate
D-1) toda vez que rodavam, rebatendo na API do JMS pra cada dia antigo.
No DROPOFF isso levava 15-20+ min (o endpoint de COLETADO pode passar de
100 mil linhas/dia) e so pioraria conforme o mes avancasse. Agora cada
execucao busca so o dia novo, salva em dados/historico_*.json, e o painel
mensal (Consolidado + Geral Diario) e montado a partir desse arquivo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/DROPOFF_diario.xlsx
+++ b/output/DROPOFF_diario.xlsx
@@ -509,13 +509,13 @@
         <v>64</v>
       </c>
       <c r="D3" t="n">
-        <v>2232</v>
+        <v>2264</v>
       </c>
       <c r="E3" t="n">
-        <v>2296</v>
+        <v>2328</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.9721</v>
+        <v>0.9725</v>
       </c>
     </row>
     <row r="4">
@@ -533,10 +533,10 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>3365</v>
+        <v>3370</v>
       </c>
       <c r="E4" t="n">
-        <v>3365</v>
+        <v>3370</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>1</v>
@@ -579,10 +579,10 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>2736</v>
+        <v>2740</v>
       </c>
       <c r="E6" t="n">
-        <v>2738</v>
+        <v>2742</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>0.9993000000000001</v>
@@ -691,13 +691,13 @@
         <v>423</v>
       </c>
       <c r="D11" t="n">
-        <v>2053</v>
+        <v>2059</v>
       </c>
       <c r="E11" t="n">
-        <v>2476</v>
+        <v>2482</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.8292</v>
+        <v>0.8295999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -737,10 +737,10 @@
         <v>40</v>
       </c>
       <c r="D13" t="n">
-        <v>3589</v>
+        <v>3595</v>
       </c>
       <c r="E13" t="n">
-        <v>3629</v>
+        <v>3635</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>0.9890000000000001</v>
@@ -761,10 +761,10 @@
         <v>42</v>
       </c>
       <c r="D14" t="n">
-        <v>6764</v>
+        <v>6779</v>
       </c>
       <c r="E14" t="n">
-        <v>6806</v>
+        <v>6821</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>0.9937999999999999</v>

</xml_diff>

<commit_message>
Atualiza historico e planilhas (run automatico)
</commit_message>
<xml_diff>
--- a/output/DROPOFF_diario.xlsx
+++ b/output/DROPOFF_diario.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxa de Coletas por Base" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Taxa de Coletas por Base" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Taxa de Coletas por Base'!$A$1:$F$15</definedName>
@@ -506,16 +506,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="D3" t="n">
-        <v>2264</v>
+        <v>2261</v>
       </c>
       <c r="E3" t="n">
-        <v>2328</v>
+        <v>2296</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.9725</v>
+        <v>0.9848</v>
       </c>
     </row>
     <row r="4">
@@ -533,10 +533,10 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>3370</v>
+        <v>3365</v>
       </c>
       <c r="E4" t="n">
-        <v>3370</v>
+        <v>3365</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>1</v>
@@ -576,16 +576,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>2740</v>
+        <v>2738</v>
       </c>
       <c r="E6" t="n">
-        <v>2742</v>
+        <v>2738</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.9993000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -688,13 +688,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D11" t="n">
-        <v>2059</v>
+        <v>2054</v>
       </c>
       <c r="E11" t="n">
-        <v>2482</v>
+        <v>2476</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>0.8295999999999999</v>
@@ -734,16 +734,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>3595</v>
+        <v>3626</v>
       </c>
       <c r="E13" t="n">
-        <v>3635</v>
+        <v>3629</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.9890000000000001</v>
+        <v>0.9992</v>
       </c>
     </row>
     <row r="14">
@@ -761,10 +761,10 @@
         <v>42</v>
       </c>
       <c r="D14" t="n">
-        <v>6779</v>
+        <v>6764</v>
       </c>
       <c r="E14" t="n">
-        <v>6821</v>
+        <v>6806</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>0.9937999999999999</v>

</xml_diff>

<commit_message>
Atualiza historico e planilhas DROPOFF (run automatico)
</commit_message>
<xml_diff>
--- a/output/DROPOFF_diario.xlsx
+++ b/output/DROPOFF_diario.xlsx
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -506,22 +506,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>35</v>
+        <v>381</v>
       </c>
       <c r="D3" t="n">
-        <v>2261</v>
+        <v>782</v>
       </c>
       <c r="E3" t="n">
-        <v>2296</v>
+        <v>1163</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.9848</v>
+        <v>0.6724</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -530,22 +530,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>3365</v>
+        <v>3200</v>
       </c>
       <c r="E4" t="n">
-        <v>3365</v>
+        <v>3228</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1</v>
+        <v>0.9913</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -567,7 +567,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -579,10 +579,10 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>2738</v>
+        <v>2643</v>
       </c>
       <c r="E6" t="n">
-        <v>2738</v>
+        <v>2643</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>1</v>
@@ -591,7 +591,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -613,7 +613,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -657,7 +657,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -666,20 +666,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>93</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="2" t="n"/>
+        <v>94</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0.9893999999999999</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -688,22 +690,22 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>422</v>
+        <v>40</v>
       </c>
       <c r="D11" t="n">
-        <v>2054</v>
+        <v>1938</v>
       </c>
       <c r="E11" t="n">
-        <v>2476</v>
+        <v>1978</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.8295999999999999</v>
+        <v>0.9798</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -725,7 +727,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -734,22 +736,22 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>3626</v>
+        <v>3212</v>
       </c>
       <c r="E13" t="n">
-        <v>3629</v>
+        <v>3216</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.9992</v>
+        <v>0.9987999999999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -758,22 +760,22 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>6764</v>
+        <v>4846</v>
       </c>
       <c r="E14" t="n">
-        <v>6806</v>
+        <v>4848</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.9937999999999999</v>
+        <v>0.9995999999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">

</xml_diff>

<commit_message>
Backfill PICKUP/DROPOFF (28-29/08) e TRANSFERENCIA (28-29/08)
Cron falhou nesses dias por token JMS expirado; backfill manual apos
renovar o token.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/DROPOFF_diario.xlsx
+++ b/output/DROPOFF_diario.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Taxa de Coletas por Base" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxa de Coletas por Base" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Taxa de Coletas por Base'!$A$1:$F$15</definedName>
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -509,17 +509,19 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>356</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="2" t="n"/>
+        <v>356</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -531,17 +533,19 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>527</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="2" t="n"/>
+        <v>527</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -563,7 +567,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -572,20 +576,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>442</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="2" t="n"/>
+        <v>443</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0.9976999999999999</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -594,20 +600,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="2" t="n"/>
+        <v>7</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -616,20 +624,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>382</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="2" t="n"/>
+        <v>382</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -638,20 +648,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="2" t="n"/>
+        <v>7</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -660,20 +672,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>497</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="2" t="n"/>
+        <v>501</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0.992</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -685,17 +699,19 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="2" t="n"/>
+        <v>14</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -717,7 +733,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -726,20 +742,22 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>535</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="2" t="n"/>
+        <v>538</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.9944</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -748,20 +766,22 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>269</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1202</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2" t="n"/>
+        <v>1471</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>0.8170999999999999</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">

</xml_diff>